<commit_message>
docs: Adding data necessary to run DEV notebook
</commit_message>
<xml_diff>
--- a/notebooks/tidysdmx/data/WB_ASPIRE_MAPPING_SUBSET.xlsx
+++ b/notebooks/tidysdmx/data/WB_ASPIRE_MAPPING_SUBSET.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\WBG\wb-projects\my-packages\tidysdmx\notebooks\tidysdmx\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2195DC8-DE39-437F-8A37-B5A80BC1D5A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3FCC7BCB-18D4-4155-8496-774756D3D353}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="266" uniqueCount="175">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="266" uniqueCount="176">
   <si>
     <t>DATA CURATION PROCESS</t>
   </si>
@@ -571,6 +571,9 @@
   </si>
   <si>
     <t>PER_ALLSP_ADQ_EP_TOT</t>
+  </si>
+  <si>
+    <t>INV</t>
   </si>
 </sst>
 </file>
@@ -1645,7 +1648,7 @@
         <v>38</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>39</v>
+        <v>175</v>
       </c>
       <c r="F3" t="s">
         <v>39</v>
@@ -1663,7 +1666,7 @@
         <v>64</v>
       </c>
       <c r="K3" s="1" t="s">
-        <v>43</v>
+        <v>175</v>
       </c>
       <c r="L3" s="23" t="s">
         <v>44</v>
@@ -13281,11 +13284,35 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<spe:Receivers xmlns:spe="http://schemas.microsoft.com/sharepoint/events"/>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="3e02667f-0271-471b-bd6e-11a2e16def1d" xsi:nil="true"/>
+    <o1cb080a3dca4eb8a0fd03c7cc8bf8f7 xmlns="3e02667f-0271-471b-bd6e-11a2e16def1d">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </o1cb080a3dca4eb8a0fd03c7cc8bf8f7>
+    <Abstract xmlns="3e02667f-0271-471b-bd6e-11a2e16def1d" xsi:nil="true"/>
+    <WBDocs_Access_To_Info_Exception xmlns="3e02667f-0271-471b-bd6e-11a2e16def1d">12. Not Assessed</WBDocs_Access_To_Info_Exception>
+    <WBDocs_Document_Date xmlns="3e02667f-0271-471b-bd6e-11a2e16def1d">2025-10-21T21:35:45+00:00</WBDocs_Document_Date>
+    <OneCMS_Subcategory xmlns="3e02667f-0271-471b-bd6e-11a2e16def1d" xsi:nil="true"/>
+    <i008215bacac45029ee8cafff4c8e93b xmlns="3e02667f-0271-471b-bd6e-11a2e16def1d">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </i008215bacac45029ee8cafff4c8e93b>
+    <WBDocs_Information_Classification xmlns="3e02667f-0271-471b-bd6e-11a2e16def1d">Official Use Only</WBDocs_Information_Classification>
+    <OneCMS_Category xmlns="3e02667f-0271-471b-bd6e-11a2e16def1d" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="WBDocument" ma:contentTypeID="0x010100F4C63C3BD852AE468EAEFD0E6C57C64F02001136FB570B32BB418C98962D1FA9A76C" ma:contentTypeVersion="4" ma:contentTypeDescription="" ma:contentTypeScope="" ma:versionID="cae7650b3b7a33991c2476527bf8bd0d">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="3e02667f-0271-471b-bd6e-11a2e16def1d" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="4226bc10e1731834a7dbc31102029e13" ns3:_="">
     <xsd:import namespace="3e02667f-0271-471b-bd6e-11a2e16def1d"/>
@@ -13527,33 +13554,9 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item5.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item5.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="3e02667f-0271-471b-bd6e-11a2e16def1d" xsi:nil="true"/>
-    <o1cb080a3dca4eb8a0fd03c7cc8bf8f7 xmlns="3e02667f-0271-471b-bd6e-11a2e16def1d">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </o1cb080a3dca4eb8a0fd03c7cc8bf8f7>
-    <Abstract xmlns="3e02667f-0271-471b-bd6e-11a2e16def1d" xsi:nil="true"/>
-    <WBDocs_Access_To_Info_Exception xmlns="3e02667f-0271-471b-bd6e-11a2e16def1d">12. Not Assessed</WBDocs_Access_To_Info_Exception>
-    <WBDocs_Document_Date xmlns="3e02667f-0271-471b-bd6e-11a2e16def1d">2025-10-21T21:35:45+00:00</WBDocs_Document_Date>
-    <OneCMS_Subcategory xmlns="3e02667f-0271-471b-bd6e-11a2e16def1d" xsi:nil="true"/>
-    <i008215bacac45029ee8cafff4c8e93b xmlns="3e02667f-0271-471b-bd6e-11a2e16def1d">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </i008215bacac45029ee8cafff4c8e93b>
-    <WBDocs_Information_Classification xmlns="3e02667f-0271-471b-bd6e-11a2e16def1d">Official Use Only</WBDocs_Information_Classification>
-    <OneCMS_Category xmlns="3e02667f-0271-471b-bd6e-11a2e16def1d" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<spe:Receivers xmlns:spe="http://schemas.microsoft.com/sharepoint/events"/>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -13565,14 +13568,24 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1C761402-8420-4FA0-A37F-4FD24EAC1096}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A981F82B-C04A-491F-B979-EFA7E42A5585}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/events"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="3e02667f-0271-471b-bd6e-11a2e16def1d"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EE6FB4C7-72EC-478A-A248-DA16B79B4830}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CF690736-D8F4-4083-807F-CA00EAA2F085}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -13590,20 +13603,10 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EE6FB4C7-72EC-478A-A248-DA16B79B4830}">
+<file path=customXml/itemProps5.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1C761402-8420-4FA0-A37F-4FD24EAC1096}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps5.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A981F82B-C04A-491F-B979-EFA7E42A5585}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="3e02667f-0271-471b-bd6e-11a2e16def1d"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/events"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
doc: update DEV notebook
</commit_message>
<xml_diff>
--- a/notebooks/tidysdmx/data/WB_ASPIRE_MAPPING_SUBSET.xlsx
+++ b/notebooks/tidysdmx/data/WB_ASPIRE_MAPPING_SUBSET.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\WBG\wb-projects\my-packages\tidysdmx\notebooks\tidysdmx\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3FCC7BCB-18D4-4155-8496-774756D3D353}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{3F95206C-A1B9-467F-AA52-BA43A896BA6D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="INFO" sheetId="11" r:id="rId1"/>
@@ -23,7 +23,7 @@
     <sheet name="INDICATOR_REF_METADATA" sheetId="12" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">REP_MAPPING!$A$1:$T$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">REP_MAPPING!$A$1:$U$3</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="266" uniqueCount="176">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="301" uniqueCount="182">
   <si>
     <t>DATA CURATION PROCESS</t>
   </si>
@@ -574,6 +574,24 @@
   </si>
   <si>
     <t>INV</t>
+  </si>
+  <si>
+    <t>S:TIME_PERIOD</t>
+  </si>
+  <si>
+    <t>2021</t>
+  </si>
+  <si>
+    <t>2018</t>
+  </si>
+  <si>
+    <t>SERIES|TIME_PERIOD</t>
+  </si>
+  <si>
+    <t>multi_representation</t>
+  </si>
+  <si>
+    <t>DEFAULT_VALUE</t>
   </si>
 </sst>
 </file>
@@ -796,10 +814,10 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyFont="1"/>
     <xf numFmtId="49" fontId="7" fillId="0" borderId="1" xfId="1" applyNumberFormat="1"/>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="49" fontId="9" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="13" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1288,15 +1306,16 @@
   <sheetPr>
     <tabColor rgb="FF00B050"/>
   </sheetPr>
-  <dimension ref="A1:C20"/>
+  <dimension ref="A1:D20"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="16.33203125" customWidth="1"/>
+    <col min="1" max="1" width="21.6640625" customWidth="1"/>
     <col min="2" max="2" width="17.6640625" customWidth="1"/>
-    <col min="3" max="3" width="16.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="21.88671875" customWidth="1"/>
+    <col min="4" max="4" width="16.21875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="4" t="s">
         <v>8</v>
       </c>
@@ -1306,8 +1325,11 @@
       <c r="C1" s="4" t="s">
         <v>162</v>
       </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D1" s="4" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>170</v>
       </c>
@@ -1318,7 +1340,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>170</v>
       </c>
@@ -1329,7 +1351,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>170</v>
       </c>
@@ -1340,7 +1362,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" s="16" t="s">
         <v>171</v>
       </c>
@@ -1351,7 +1373,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>170</v>
       </c>
@@ -1362,7 +1384,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>170</v>
       </c>
@@ -1373,7 +1395,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>170</v>
       </c>
@@ -1384,7 +1406,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>170</v>
       </c>
@@ -1395,7 +1417,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>170</v>
       </c>
@@ -1406,18 +1428,21 @@
         <v>167</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>170</v>
+        <v>179</v>
       </c>
       <c r="B11" s="20" t="s">
         <v>165</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>167</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+        <v>180</v>
+      </c>
+      <c r="D11" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B12" s="20" t="s">
         <v>30</v>
       </c>
@@ -1425,7 +1450,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
         <v>172</v>
       </c>
@@ -1436,7 +1461,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="s">
         <v>31</v>
       </c>
@@ -1447,7 +1472,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B15" s="20" t="s">
         <v>32</v>
       </c>
@@ -1455,7 +1480,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B16" s="20" t="s">
         <v>33</v>
       </c>
@@ -1503,207 +1528,334 @@
   <sheetPr>
     <tabColor theme="9"/>
   </sheetPr>
-  <dimension ref="A1:T3"/>
+  <dimension ref="A1:U5"/>
   <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="43.109375" style="2" customWidth="1"/>
-    <col min="2" max="2" width="36.6640625" style="2" customWidth="1"/>
-    <col min="3" max="3" width="19.44140625" style="2" customWidth="1"/>
-    <col min="4" max="9" width="19.5546875" style="2" customWidth="1"/>
-    <col min="10" max="10" width="21.109375" style="2" customWidth="1"/>
-    <col min="11" max="11" width="21.88671875" style="2" customWidth="1"/>
-    <col min="12" max="12" width="8.6640625" style="2"/>
-    <col min="13" max="13" width="14" style="2" customWidth="1"/>
-    <col min="14" max="16" width="8.6640625" style="2"/>
-    <col min="17" max="17" width="8.6640625" style="24"/>
-    <col min="18" max="16384" width="8.6640625" style="2"/>
+    <col min="1" max="2" width="43.109375" style="2" customWidth="1"/>
+    <col min="3" max="3" width="36.6640625" style="2" customWidth="1"/>
+    <col min="4" max="4" width="19.44140625" style="2" customWidth="1"/>
+    <col min="5" max="10" width="19.5546875" style="2" customWidth="1"/>
+    <col min="11" max="11" width="21.109375" style="2" customWidth="1"/>
+    <col min="12" max="12" width="21.88671875" style="2" customWidth="1"/>
+    <col min="13" max="13" width="8.6640625" style="2"/>
+    <col min="14" max="14" width="14" style="2" customWidth="1"/>
+    <col min="15" max="17" width="8.6640625" style="2"/>
+    <col min="18" max="18" width="8.6640625" style="24"/>
+    <col min="19" max="16384" width="8.6640625" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:21" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
         <v>168</v>
       </c>
       <c r="B1" s="3" t="s">
+        <v>176</v>
+      </c>
+      <c r="C1" s="3" t="s">
         <v>169</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="D1" s="3" t="s">
         <v>145</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="E1" s="3" t="s">
         <v>146</v>
       </c>
-      <c r="E1" s="17" t="s">
+      <c r="F1" s="17" t="s">
         <v>147</v>
       </c>
-      <c r="F1" s="17" t="s">
+      <c r="G1" s="17" t="s">
         <v>148</v>
       </c>
-      <c r="G1" s="17" t="s">
+      <c r="H1" s="17" t="s">
         <v>149</v>
       </c>
-      <c r="H1" s="17" t="s">
+      <c r="I1" s="17" t="s">
         <v>150</v>
       </c>
-      <c r="I1" s="17" t="s">
+      <c r="J1" s="17" t="s">
         <v>151</v>
       </c>
-      <c r="J1" s="17" t="s">
+      <c r="K1" s="17" t="s">
         <v>152</v>
       </c>
-      <c r="K1" s="3" t="s">
+      <c r="L1" s="3" t="s">
         <v>153</v>
       </c>
-      <c r="L1" s="3" t="s">
+      <c r="M1" s="3" t="s">
         <v>154</v>
       </c>
-      <c r="M1" s="3" t="s">
+      <c r="N1" s="3" t="s">
         <v>155</v>
       </c>
-      <c r="N1" s="3" t="s">
+      <c r="O1" s="3" t="s">
         <v>156</v>
       </c>
-      <c r="O1" s="3" t="s">
+      <c r="P1" s="3" t="s">
         <v>157</v>
       </c>
-      <c r="P1" s="3" t="s">
+      <c r="Q1" s="3" t="s">
         <v>158</v>
       </c>
-      <c r="Q1" s="26" t="s">
+      <c r="R1" s="25" t="s">
         <v>166</v>
       </c>
-      <c r="R1" s="3" t="s">
+      <c r="S1" s="3" t="s">
         <v>159</v>
       </c>
-      <c r="S1" s="3" t="s">
+      <c r="T1" s="3" t="s">
         <v>160</v>
       </c>
-      <c r="T1" s="3" t="s">
+      <c r="U1" s="3" t="s">
         <v>161</v>
       </c>
     </row>
-    <row r="2" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>173</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2">
+        <v>2021</v>
+      </c>
+      <c r="C2" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="E2" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="F2" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="F2" t="s">
+      <c r="G2" t="s">
         <v>39</v>
       </c>
-      <c r="G2" s="1" t="s">
+      <c r="H2" s="1" t="s">
         <v>164</v>
       </c>
-      <c r="H2" t="s">
+      <c r="I2" t="s">
         <v>66</v>
       </c>
-      <c r="I2" s="1" t="s">
+      <c r="J2" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="J2" t="s">
+      <c r="K2" t="s">
         <v>64</v>
       </c>
-      <c r="K2" s="1" t="s">
+      <c r="L2" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="L2" s="23" t="s">
+      <c r="M2" s="23" t="s">
         <v>44</v>
       </c>
-      <c r="N2" s="23" t="s">
+      <c r="O2" s="23" t="s">
         <v>45</v>
       </c>
-      <c r="O2" s="23" t="s">
+      <c r="P2" s="23" t="s">
         <v>2</v>
       </c>
-      <c r="P2" s="23" t="s">
+      <c r="Q2" s="23" t="s">
         <v>46</v>
       </c>
-      <c r="Q2" s="25" t="s">
-        <v>40</v>
-      </c>
-      <c r="R2" s="2">
+      <c r="R2" s="26" t="s">
+        <v>177</v>
+      </c>
+      <c r="S2" s="2">
         <v>2</v>
       </c>
-      <c r="S2" s="2">
+      <c r="T2" s="2">
         <v>0</v>
       </c>
-      <c r="T2" s="23" t="s">
+      <c r="U2" s="23" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="3" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>174</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3">
+        <v>2021</v>
+      </c>
+      <c r="C3" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="E3" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="E3" s="1" t="s">
+      <c r="F3" s="1" t="s">
         <v>175</v>
       </c>
-      <c r="F3" t="s">
+      <c r="G3" t="s">
         <v>39</v>
       </c>
-      <c r="G3" s="1" t="s">
+      <c r="H3" s="1" t="s">
         <v>164</v>
       </c>
-      <c r="H3" t="s">
+      <c r="I3" t="s">
         <v>65</v>
       </c>
-      <c r="I3" s="1" t="s">
+      <c r="J3" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="J3" t="s">
+      <c r="K3" t="s">
         <v>64</v>
       </c>
-      <c r="K3" s="1" t="s">
+      <c r="L3" s="1" t="s">
         <v>175</v>
       </c>
-      <c r="L3" s="23" t="s">
+      <c r="M3" s="23" t="s">
         <v>44</v>
       </c>
-      <c r="N3" s="23" t="s">
+      <c r="O3" s="23" t="s">
         <v>45</v>
       </c>
-      <c r="O3" s="23" t="s">
+      <c r="P3" s="23" t="s">
         <v>2</v>
       </c>
-      <c r="P3" s="23" t="s">
+      <c r="Q3" s="23" t="s">
         <v>46</v>
       </c>
-      <c r="Q3" s="25" t="s">
-        <v>40</v>
-      </c>
-      <c r="R3" s="2">
+      <c r="R3" s="26" t="s">
+        <v>177</v>
+      </c>
+      <c r="S3" s="2">
         <v>2</v>
       </c>
-      <c r="S3" s="2">
+      <c r="T3" s="2">
         <v>0</v>
       </c>
-      <c r="T3" s="23" t="s">
+      <c r="U3" s="23" t="s">
         <v>20</v>
       </c>
     </row>
+    <row r="4" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>173</v>
+      </c>
+      <c r="B4">
+        <v>1998</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="G4" t="s">
+        <v>39</v>
+      </c>
+      <c r="H4" s="1" t="s">
+        <v>164</v>
+      </c>
+      <c r="I4" t="s">
+        <v>66</v>
+      </c>
+      <c r="J4" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="K4" t="s">
+        <v>64</v>
+      </c>
+      <c r="L4" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="M4" s="23" t="s">
+        <v>44</v>
+      </c>
+      <c r="O4" s="23" t="s">
+        <v>45</v>
+      </c>
+      <c r="P4" s="23" t="s">
+        <v>2</v>
+      </c>
+      <c r="Q4" s="23" t="s">
+        <v>46</v>
+      </c>
+      <c r="R4" s="26" t="s">
+        <v>178</v>
+      </c>
+      <c r="S4" s="2">
+        <v>2</v>
+      </c>
+      <c r="T4" s="2">
+        <v>0</v>
+      </c>
+      <c r="U4" s="23" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="5" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>174</v>
+      </c>
+      <c r="B5">
+        <v>1998</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>175</v>
+      </c>
+      <c r="G5" t="s">
+        <v>39</v>
+      </c>
+      <c r="H5" s="1" t="s">
+        <v>164</v>
+      </c>
+      <c r="I5" t="s">
+        <v>65</v>
+      </c>
+      <c r="J5" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="K5" t="s">
+        <v>64</v>
+      </c>
+      <c r="L5" s="1" t="s">
+        <v>175</v>
+      </c>
+      <c r="M5" s="23" t="s">
+        <v>44</v>
+      </c>
+      <c r="O5" s="23" t="s">
+        <v>45</v>
+      </c>
+      <c r="P5" s="23" t="s">
+        <v>2</v>
+      </c>
+      <c r="Q5" s="23" t="s">
+        <v>46</v>
+      </c>
+      <c r="R5" s="26" t="s">
+        <v>178</v>
+      </c>
+      <c r="S5" s="2">
+        <v>2</v>
+      </c>
+      <c r="T5" s="2">
+        <v>0</v>
+      </c>
+      <c r="U5" s="23" t="s">
+        <v>20</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:T3" xr:uid="{B2B9A685-B78A-41EF-9688-4C3FB8FF0CD6}">
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:T3">
+  <autoFilter ref="A1:U3" xr:uid="{B2B9A685-B78A-41EF-9688-4C3FB8FF0CD6}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:U3">
       <sortCondition ref="A1:A3"/>
     </sortState>
   </autoFilter>
   <phoneticPr fontId="11" type="noConversion"/>
-  <conditionalFormatting sqref="A4:A1048576 A1">
+  <conditionalFormatting sqref="A6:B1048576 A1">
     <cfRule type="duplicateValues" dxfId="1" priority="10"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C2:C3">
+  <conditionalFormatting sqref="D2:D5">
     <cfRule type="duplicateValues" dxfId="0" priority="12"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -13284,35 +13436,11 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="3e02667f-0271-471b-bd6e-11a2e16def1d" xsi:nil="true"/>
-    <o1cb080a3dca4eb8a0fd03c7cc8bf8f7 xmlns="3e02667f-0271-471b-bd6e-11a2e16def1d">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </o1cb080a3dca4eb8a0fd03c7cc8bf8f7>
-    <Abstract xmlns="3e02667f-0271-471b-bd6e-11a2e16def1d" xsi:nil="true"/>
-    <WBDocs_Access_To_Info_Exception xmlns="3e02667f-0271-471b-bd6e-11a2e16def1d">12. Not Assessed</WBDocs_Access_To_Info_Exception>
-    <WBDocs_Document_Date xmlns="3e02667f-0271-471b-bd6e-11a2e16def1d">2025-10-21T21:35:45+00:00</WBDocs_Document_Date>
-    <OneCMS_Subcategory xmlns="3e02667f-0271-471b-bd6e-11a2e16def1d" xsi:nil="true"/>
-    <i008215bacac45029ee8cafff4c8e93b xmlns="3e02667f-0271-471b-bd6e-11a2e16def1d">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </i008215bacac45029ee8cafff4c8e93b>
-    <WBDocs_Information_Classification xmlns="3e02667f-0271-471b-bd6e-11a2e16def1d">Official Use Only</WBDocs_Information_Classification>
-    <OneCMS_Category xmlns="3e02667f-0271-471b-bd6e-11a2e16def1d" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<spe:Receivers xmlns:spe="http://schemas.microsoft.com/sharepoint/events"/>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="WBDocument" ma:contentTypeID="0x010100F4C63C3BD852AE468EAEFD0E6C57C64F02001136FB570B32BB418C98962D1FA9A76C" ma:contentTypeVersion="4" ma:contentTypeDescription="" ma:contentTypeScope="" ma:versionID="cae7650b3b7a33991c2476527bf8bd0d">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="3e02667f-0271-471b-bd6e-11a2e16def1d" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="4226bc10e1731834a7dbc31102029e13" ns3:_="">
     <xsd:import namespace="3e02667f-0271-471b-bd6e-11a2e16def1d"/>
@@ -13554,9 +13682,33 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/item5.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<spe:Receivers xmlns:spe="http://schemas.microsoft.com/sharepoint/events"/>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="3e02667f-0271-471b-bd6e-11a2e16def1d" xsi:nil="true"/>
+    <o1cb080a3dca4eb8a0fd03c7cc8bf8f7 xmlns="3e02667f-0271-471b-bd6e-11a2e16def1d">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </o1cb080a3dca4eb8a0fd03c7cc8bf8f7>
+    <Abstract xmlns="3e02667f-0271-471b-bd6e-11a2e16def1d" xsi:nil="true"/>
+    <WBDocs_Access_To_Info_Exception xmlns="3e02667f-0271-471b-bd6e-11a2e16def1d">12. Not Assessed</WBDocs_Access_To_Info_Exception>
+    <WBDocs_Document_Date xmlns="3e02667f-0271-471b-bd6e-11a2e16def1d">2025-10-21T21:35:45+00:00</WBDocs_Document_Date>
+    <OneCMS_Subcategory xmlns="3e02667f-0271-471b-bd6e-11a2e16def1d" xsi:nil="true"/>
+    <i008215bacac45029ee8cafff4c8e93b xmlns="3e02667f-0271-471b-bd6e-11a2e16def1d">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </i008215bacac45029ee8cafff4c8e93b>
+    <WBDocs_Information_Classification xmlns="3e02667f-0271-471b-bd6e-11a2e16def1d">Official Use Only</WBDocs_Information_Classification>
+    <OneCMS_Category xmlns="3e02667f-0271-471b-bd6e-11a2e16def1d" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -13568,24 +13720,14 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A981F82B-C04A-491F-B979-EFA7E42A5585}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1C761402-8420-4FA0-A37F-4FD24EAC1096}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="3e02667f-0271-471b-bd6e-11a2e16def1d"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/events"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EE6FB4C7-72EC-478A-A248-DA16B79B4830}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CF690736-D8F4-4083-807F-CA00EAA2F085}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -13603,10 +13745,20 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EE6FB4C7-72EC-478A-A248-DA16B79B4830}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps5.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1C761402-8420-4FA0-A37F-4FD24EAC1096}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A981F82B-C04A-491F-B979-EFA7E42A5585}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/events"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="3e02667f-0271-471b-bd6e-11a2e16def1d"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
feat: improve sdmx artefacts publication flow
</commit_message>
<xml_diff>
--- a/notebooks/tidysdmx/data/WB_ASPIRE_MAPPING_SUBSET.xlsx
+++ b/notebooks/tidysdmx/data/WB_ASPIRE_MAPPING_SUBSET.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
-  <workbookPr/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\WBG\wb-projects\my-packages\tidysdmx\notebooks\tidysdmx\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{3F95206C-A1B9-467F-AA52-BA43A896BA6D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{202F8206-F859-4B02-B247-BCF63396C705}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="INFO" sheetId="11" r:id="rId1"/>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="301" uniqueCount="182">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="301" uniqueCount="181">
   <si>
     <t>DATA CURATION PROCESS</t>
   </si>
@@ -571,9 +571,6 @@
   </si>
   <si>
     <t>PER_ALLSP_ADQ_EP_TOT</t>
-  </si>
-  <si>
-    <t>INV</t>
   </si>
   <si>
     <t>S:TIME_PERIOD</t>
@@ -1326,7 +1323,7 @@
         <v>162</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
@@ -1430,13 +1427,13 @@
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="B11" s="20" t="s">
         <v>165</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="D11" t="s">
         <v>40</v>
@@ -1549,7 +1546,7 @@
         <v>168</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="C1" s="3" t="s">
         <v>169</v>
@@ -1656,7 +1653,7 @@
         <v>46</v>
       </c>
       <c r="R2" s="26" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="S2" s="2">
         <v>2</v>
@@ -1682,7 +1679,7 @@
         <v>38</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>175</v>
+        <v>39</v>
       </c>
       <c r="G3" t="s">
         <v>39</v>
@@ -1700,7 +1697,7 @@
         <v>64</v>
       </c>
       <c r="L3" s="1" t="s">
-        <v>175</v>
+        <v>43</v>
       </c>
       <c r="M3" s="23" t="s">
         <v>44</v>
@@ -1715,7 +1712,7 @@
         <v>46</v>
       </c>
       <c r="R3" s="26" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="S3" s="2">
         <v>2</v>
@@ -1774,7 +1771,7 @@
         <v>46</v>
       </c>
       <c r="R4" s="26" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="S4" s="2">
         <v>2</v>
@@ -1800,7 +1797,7 @@
         <v>38</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>175</v>
+        <v>39</v>
       </c>
       <c r="G5" t="s">
         <v>39</v>
@@ -1818,7 +1815,7 @@
         <v>64</v>
       </c>
       <c r="L5" s="1" t="s">
-        <v>175</v>
+        <v>43</v>
       </c>
       <c r="M5" s="23" t="s">
         <v>44</v>
@@ -1833,7 +1830,7 @@
         <v>46</v>
       </c>
       <c r="R5" s="26" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="S5" s="2">
         <v>2</v>
@@ -13436,11 +13433,35 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<spe:Receivers xmlns:spe="http://schemas.microsoft.com/sharepoint/events"/>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="3e02667f-0271-471b-bd6e-11a2e16def1d" xsi:nil="true"/>
+    <o1cb080a3dca4eb8a0fd03c7cc8bf8f7 xmlns="3e02667f-0271-471b-bd6e-11a2e16def1d">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </o1cb080a3dca4eb8a0fd03c7cc8bf8f7>
+    <Abstract xmlns="3e02667f-0271-471b-bd6e-11a2e16def1d" xsi:nil="true"/>
+    <WBDocs_Access_To_Info_Exception xmlns="3e02667f-0271-471b-bd6e-11a2e16def1d">12. Not Assessed</WBDocs_Access_To_Info_Exception>
+    <WBDocs_Document_Date xmlns="3e02667f-0271-471b-bd6e-11a2e16def1d">2025-10-21T21:35:45+00:00</WBDocs_Document_Date>
+    <OneCMS_Subcategory xmlns="3e02667f-0271-471b-bd6e-11a2e16def1d" xsi:nil="true"/>
+    <i008215bacac45029ee8cafff4c8e93b xmlns="3e02667f-0271-471b-bd6e-11a2e16def1d">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </i008215bacac45029ee8cafff4c8e93b>
+    <WBDocs_Information_Classification xmlns="3e02667f-0271-471b-bd6e-11a2e16def1d">Official Use Only</WBDocs_Information_Classification>
+    <OneCMS_Category xmlns="3e02667f-0271-471b-bd6e-11a2e16def1d" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="WBDocument" ma:contentTypeID="0x010100F4C63C3BD852AE468EAEFD0E6C57C64F02001136FB570B32BB418C98962D1FA9A76C" ma:contentTypeVersion="4" ma:contentTypeDescription="" ma:contentTypeScope="" ma:versionID="cae7650b3b7a33991c2476527bf8bd0d">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="3e02667f-0271-471b-bd6e-11a2e16def1d" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="4226bc10e1731834a7dbc31102029e13" ns3:_="">
     <xsd:import namespace="3e02667f-0271-471b-bd6e-11a2e16def1d"/>
@@ -13682,33 +13703,9 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item5.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item5.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="3e02667f-0271-471b-bd6e-11a2e16def1d" xsi:nil="true"/>
-    <o1cb080a3dca4eb8a0fd03c7cc8bf8f7 xmlns="3e02667f-0271-471b-bd6e-11a2e16def1d">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </o1cb080a3dca4eb8a0fd03c7cc8bf8f7>
-    <Abstract xmlns="3e02667f-0271-471b-bd6e-11a2e16def1d" xsi:nil="true"/>
-    <WBDocs_Access_To_Info_Exception xmlns="3e02667f-0271-471b-bd6e-11a2e16def1d">12. Not Assessed</WBDocs_Access_To_Info_Exception>
-    <WBDocs_Document_Date xmlns="3e02667f-0271-471b-bd6e-11a2e16def1d">2025-10-21T21:35:45+00:00</WBDocs_Document_Date>
-    <OneCMS_Subcategory xmlns="3e02667f-0271-471b-bd6e-11a2e16def1d" xsi:nil="true"/>
-    <i008215bacac45029ee8cafff4c8e93b xmlns="3e02667f-0271-471b-bd6e-11a2e16def1d">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </i008215bacac45029ee8cafff4c8e93b>
-    <WBDocs_Information_Classification xmlns="3e02667f-0271-471b-bd6e-11a2e16def1d">Official Use Only</WBDocs_Information_Classification>
-    <OneCMS_Category xmlns="3e02667f-0271-471b-bd6e-11a2e16def1d" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<spe:Receivers xmlns:spe="http://schemas.microsoft.com/sharepoint/events"/>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -13720,14 +13717,24 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1C761402-8420-4FA0-A37F-4FD24EAC1096}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A981F82B-C04A-491F-B979-EFA7E42A5585}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/events"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="3e02667f-0271-471b-bd6e-11a2e16def1d"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EE6FB4C7-72EC-478A-A248-DA16B79B4830}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CF690736-D8F4-4083-807F-CA00EAA2F085}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -13745,20 +13752,10 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EE6FB4C7-72EC-478A-A248-DA16B79B4830}">
+<file path=customXml/itemProps5.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1C761402-8420-4FA0-A37F-4FD24EAC1096}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps5.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A981F82B-C04A-491F-B979-EFA7E42A5585}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="3e02667f-0271-471b-bd6e-11a2e16def1d"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/events"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>